<commit_message>
feat(customer,recharging,charger): 동/호 컬럼 분리 및 목록 UI 개선
- TB_CUCU001.DONG_HO를 DONG/HO로 분리 (ALTER_DONG_HO_SPLIT.sql), 관련 매퍼/도메인 전면 수정
- customerList: 정렬 select를 라디오(가입일/고객명 asc/desc)로 변경, 컬럼을 단지/동/호 등으로 재구성
- rechargingList, rechargingCustomerList, statusInfoList: 동/호를 별도 컬럼으로 분리 표출
- rechargingCustomerList: 순번(번호) 컬럼 추가
- ChargerStatusResource: 예외 스택트레이스 로깅 추가
- TB_CUCU002 인증 관련 컬럼 복구 스크립트 추가 (ALTER_RESTORE_MEMBER_AUTH_COLS.sql)
</commit_message>
<xml_diff>
--- a/localcsms/web/admin-web/src/main/resources/CP_001.xlsx
+++ b/localcsms/web/admin-web/src/main/resources/CP_001.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26529"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\igKang\workspace\kevit-LocalCsmsWeb_workspace\local-csms\localcsms\web\admin-web\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AntigravityProject\lh\localcsms\web\admin-web\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A8E475-5601-463A-8A93-B6F53B5DCE53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D243276-42BD-425D-B104-919DDAED8DF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-32640" yWindow="5760" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4068" yWindow="4188" windowWidth="34560" windowHeight="18600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -43,16 +43,12 @@
   </si>
   <si>
     <t>충전소 목록</t>
-    <phoneticPr fontId="4" type="noConversion"/>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>충전소ID</t>
   </si>
   <si>
-    <t>순번</t>
-    <phoneticPr fontId="0" type="noConversion"/>
-  </si>
-  <si>
     <t>사용 여부</t>
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
@@ -93,6 +89,10 @@
   </si>
   <si>
     <t>${excelData.lowCsCount}</t>
+    <phoneticPr fontId="0" type="noConversion"/>
+  </si>
+  <si>
+    <t>No.</t>
     <phoneticPr fontId="0" type="noConversion"/>
   </si>
 </sst>
@@ -105,7 +105,7 @@
     <numFmt numFmtId="177" formatCode="0.00_);\(0.00\)"/>
     <numFmt numFmtId="178" formatCode="0_);\(0\)"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -119,26 +119,7 @@
       <charset val="204"/>
     </font>
     <font>
-      <b/>
-      <sz val="12"/>
-      <name val="돋움"/>
-      <family val="3"/>
-      <charset val="129"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="204"/>
-    </font>
-    <font>
       <sz val="8"/>
-      <name val="돋움"/>
-      <family val="3"/>
-      <charset val="129"/>
-    </font>
-    <font>
-      <sz val="20"/>
       <name val="돋움"/>
       <family val="3"/>
       <charset val="129"/>
@@ -146,9 +127,39 @@
     <font>
       <b/>
       <sz val="20"/>
-      <name val="돋움"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -267,49 +278,49 @@
   </cellStyleXfs>
   <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="6" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="6" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -618,106 +629,106 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I5"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.140625" style="10" customWidth="1"/>
-    <col min="3" max="3" width="25.5703125" style="10" customWidth="1"/>
-    <col min="4" max="4" width="33.5703125" style="10" customWidth="1"/>
-    <col min="5" max="5" width="23.5703125" style="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.85546875" style="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.5703125" style="10" customWidth="1"/>
-    <col min="8" max="8" width="24.140625" style="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9.140625" style="10"/>
+    <col min="1" max="1" width="18.44140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="25.5546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="33.5546875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="23.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.5546875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="24.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:9" ht="30">
+      <c r="A1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2" s="15"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
-      <c r="H2" s="15"/>
-      <c r="I2" s="15"/>
+    <row r="2" spans="1:9" ht="13.2" customHeight="1">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
     </row>
-    <row r="3" spans="1:9" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:9" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+    <row r="3" spans="1:9" ht="16.2" thickBot="1"/>
+    <row r="4" spans="1:9" ht="19.2">
+      <c r="A4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="G4" s="3" t="s">
+      <c r="I4" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="18" thickBot="1">
+      <c r="A5" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="13" t="s">
+      <c r="H5" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" s="7" t="s">
+      <c r="I5" s="15" t="s">
         <v>14</v>
-      </c>
-      <c r="I5" s="12" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:I2"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>